<commit_message>
Actualizar Centro de Conocimiento
</commit_message>
<xml_diff>
--- a/data/Centro_Conocimiento_LEAN.xlsx
+++ b/data/Centro_Conocimiento_LEAN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dpherrera\Documents\CentroConocimientoLEAN\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{588AEFEF-4218-459B-B109-E65DF9F066B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87E95CA7-3404-4C0A-BB17-DB7C7ED36D05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Herramientas" sheetId="1" r:id="rId1"/>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="689" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="470">
   <si>
     <t>ID</t>
   </si>
@@ -558,9 +558,6 @@
     <t>Plan de trabajo actualizado y compromisos de planificación</t>
   </si>
   <si>
-    <t>Procedimiento de Planificación Lean</t>
-  </si>
-  <si>
     <t>PRO-002</t>
   </si>
   <si>
@@ -576,9 +573,6 @@
     <t>Plan semanal de trabajo y seguimiento de compromisos</t>
   </si>
   <si>
-    <t>Manual Last Planner System</t>
-  </si>
-  <si>
     <t>PRO-003</t>
   </si>
   <si>
@@ -594,9 +588,6 @@
     <t>Restricciones gestionadas y actualizadas</t>
   </si>
   <si>
-    <t>Procedimiento Gestión de Restricciones</t>
-  </si>
-  <si>
     <t>PRO-004</t>
   </si>
   <si>
@@ -612,9 +603,6 @@
     <t>Reportes e indicadores actualizados</t>
   </si>
   <si>
-    <t>Procedimiento de Indicadores LEAN</t>
-  </si>
-  <si>
     <t>PRO-005</t>
   </si>
   <si>
@@ -630,9 +618,6 @@
     <t>Estado actualizado de compromisos y reportes de cumplimiento</t>
   </si>
   <si>
-    <t>Procedimiento Gestión de Actas</t>
-  </si>
-  <si>
     <t>PRO-006</t>
   </si>
   <si>
@@ -648,9 +633,6 @@
     <t>Herramientas actualizadas y soporte funcional</t>
   </si>
   <si>
-    <t>Manual de Herramientas LEAN</t>
-  </si>
-  <si>
     <t>PRO-007</t>
   </si>
   <si>
@@ -666,120 +648,21 @@
     <t>Nuevos desarrollos, automatizaciones y mejoras implementadas</t>
   </si>
   <si>
-    <t>Procedimiento de Desarrollo LEAN</t>
-  </si>
-  <si>
-    <t>Manual de Analytics</t>
-  </si>
-  <si>
-    <t>Manual de Zoho Qntrl</t>
-  </si>
-  <si>
-    <t>Manual de Power BI</t>
-  </si>
-  <si>
-    <t>Procedimiento Last Planner</t>
-  </si>
-  <si>
-    <t>Guía de Preconstrucción</t>
-  </si>
-  <si>
-    <t>Instructivo Centro de Conocimiento LEAN</t>
-  </si>
-  <si>
-    <t>Formato de Actas</t>
-  </si>
-  <si>
-    <t>Formato Pull Planning</t>
-  </si>
-  <si>
-    <t>DOC-001</t>
-  </si>
-  <si>
-    <t>Manual de Usuario</t>
-  </si>
-  <si>
-    <t>SharePoint / Carpeta LEAN</t>
-  </si>
-  <si>
-    <t>1.0</t>
-  </si>
-  <si>
-    <t>DOC-002</t>
-  </si>
-  <si>
-    <t>DOC-003</t>
-  </si>
-  <si>
-    <t>Manual de Zoho Sprints</t>
-  </si>
-  <si>
-    <t>DOC-004</t>
-  </si>
-  <si>
-    <t>Procedimiento de Planificación LEAN</t>
-  </si>
-  <si>
     <t>Procedimiento</t>
   </si>
   <si>
-    <t>DOC-005</t>
-  </si>
-  <si>
-    <t>Procedimiento de Gestión de Restricciones</t>
-  </si>
-  <si>
-    <t>DOC-006</t>
-  </si>
-  <si>
     <t>Instructivo</t>
   </si>
   <si>
-    <t>Repositorio del proyecto</t>
-  </si>
-  <si>
-    <t>DOC-007</t>
-  </si>
-  <si>
-    <t>Manual Dashboard Cumplimiento de Actas</t>
-  </si>
-  <si>
-    <t>Manual Técnico</t>
-  </si>
-  <si>
-    <t>DOC-008</t>
-  </si>
-  <si>
-    <t>Manual Dashboard PPC</t>
-  </si>
-  <si>
-    <t>DOC-009</t>
-  </si>
-  <si>
-    <t>Manual Dashboard PAC</t>
-  </si>
-  <si>
-    <t>DOC-010</t>
-  </si>
-  <si>
-    <t>Formato de Actas de Reunión</t>
-  </si>
-  <si>
     <t>Formato</t>
   </si>
   <si>
-    <t>SharePoint / Formatos</t>
-  </si>
-  <si>
     <t>Coordinar la estrategia del Área LEAN y liderar iniciativas de mejora continua.</t>
   </si>
   <si>
     <t>Área LEAN</t>
   </si>
   <si>
-    <t>Ingeniera LEAN</t>
-  </si>
-  <si>
     <t>Gestionar indicadores, herramientas y procesos Lean.</t>
   </si>
   <si>
@@ -1071,33 +954,12 @@
     <t>-</t>
   </si>
   <si>
-    <t>Camilo</t>
-  </si>
-  <si>
-    <t>https://sprints.zoho.com/workspace/marval2#P163/itemdetails/I102</t>
-  </si>
-  <si>
-    <t>(239) Zoho Sprints - Item Details</t>
-  </si>
-  <si>
-    <t>https://sprints.zoho.com/workspace/marval2#P163/itemdetails/I12/description</t>
-  </si>
-  <si>
-    <t>https://sprints.zoho.com/workspace/marval2#P163/itemdetails/I129</t>
-  </si>
-  <si>
     <t>DEV-003</t>
   </si>
   <si>
     <t>DEV-004</t>
   </si>
   <si>
-    <t>DEV-005</t>
-  </si>
-  <si>
-    <t>DEV-006</t>
-  </si>
-  <si>
     <t>HER-011</t>
   </si>
   <si>
@@ -1264,13 +1126,373 @@
   </si>
   <si>
     <t>MANUAL DE CRITERIOS PARA LA IDENTIFICACIÓN DE RESTRICCIONES EN LPS</t>
+  </si>
+  <si>
+    <t>(URL):https://miro.com/app/dashboard</t>
+  </si>
+  <si>
+    <t>(URL): https://us1.aconex.com/hub/index.html</t>
+  </si>
+  <si>
+    <t>(URL): https://www.youtube.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(URL): </t>
+  </si>
+  <si>
+    <t>(URL): https://produccion.jde.marval.com.co/jde/E1Menu.maf</t>
+  </si>
+  <si>
+    <t>(URL):https://jam.dev/s/c1760f76-7d6f-4108-ba72-628a2ea1b48d</t>
+  </si>
+  <si>
+    <t>(URL): https://crmplus.zoho.com/marval3424/index.do</t>
+  </si>
+  <si>
+    <t>BA-015</t>
+  </si>
+  <si>
+    <t>BA-016</t>
+  </si>
+  <si>
+    <t>BA-023</t>
+  </si>
+  <si>
+    <t>BA-026</t>
+  </si>
+  <si>
+    <t>BA-027</t>
+  </si>
+  <si>
+    <t>BA-028</t>
+  </si>
+  <si>
+    <t>Evaluar el nivel de implementación y madurez de la metodología LEAN en las obras mediante una auditoría estructurada que permita identificar fortalezas, oportunidades de mejora y hacer seguimiento a la evolución de cada proyecto.</t>
+  </si>
+  <si>
+    <t>Integración Sellos de Calidad</t>
+  </si>
+  <si>
+    <t>Módulo que integra la gestión de Sellos de Calidad con el Avance de Grilla, permitiendo validar el cumplimiento de los criterios de calidad durante la ejecución de las actividades. Esta integración mejora la trazabilidad del proceso constructivo, evita reportes de avance sin validación y proporciona información más confiable para el seguimiento de la producción.</t>
+  </si>
+  <si>
+    <t>TICs</t>
+  </si>
+  <si>
+    <t>Módulo desarrollado para optimizar la gestión de restricciones mediante la automatización de reglas de negocio y la parametrización de actividades. Incorpora funcionalidades para la creación, administración, liberación y eliminación de restricciones, así como la edición controlada de fechas de inicio de fabricación y legalización, actualización de acuerdos de servicio, modificación de subtipos y atributos de las actividades, garantizando una programación más flexible, trazable y alineada con el proceso constructivo.</t>
+  </si>
+  <si>
+    <t>Automatización de Restricciones</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b5</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b6</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b7</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b8</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b9</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b10</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b11</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b12</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b13</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b14</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b15</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b16</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b17</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b18</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b19</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b20</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b21</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b22</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b23</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b24</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b25</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b26</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b27</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b28</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b29</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b30</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b31</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b32</t>
+  </si>
+  <si>
+    <t>Duplicidad de avances dos clicks en guardar todo en reportar avance</t>
+  </si>
+  <si>
+    <t>Por agregar</t>
+  </si>
+  <si>
+    <t>Agregar CNC en reporte preliminar</t>
+  </si>
+  <si>
+    <t>Cuando se incumple una restricción, observacion y no cumplimiento debe serobligatorio</t>
+  </si>
+  <si>
+    <t>Last Planner</t>
+  </si>
+  <si>
+    <t>Crear historia</t>
+  </si>
+  <si>
+    <t>CNC cuando se hace reducción</t>
+  </si>
+  <si>
+    <t>Avances</t>
+  </si>
+  <si>
+    <t>Implentar</t>
+  </si>
+  <si>
+    <t>Se desconecta las unidades con las tareas, activar la bandera por proyectos para hacerlo nacional (SE DEBE VALDIAR SI TIENE UNIDADES PERDIDAS, LEAN DEBE DEFINIR CUALES SON)</t>
+  </si>
+  <si>
+    <t>BA-030</t>
+  </si>
+  <si>
+    <t>BA-031</t>
+  </si>
+  <si>
+    <t>BA-032</t>
+  </si>
+  <si>
+    <t>BA-033</t>
+  </si>
+  <si>
+    <t>BA-034</t>
+  </si>
+  <si>
+    <t>Daniela</t>
+  </si>
+  <si>
+    <t>Avance fuera de reunión Last Planner (Número de caso 85972)</t>
+  </si>
+  <si>
+    <t>Caso (#85972) - AVANCE FUERA DE REUNION LAST PLANNER - GLPI</t>
+  </si>
+  <si>
+    <t>Avance por fuera de reunión Last Palnner (Número de caso 85977)</t>
+  </si>
+  <si>
+    <t>Caso (#85977) - AVANCE FUERA DE REUNION LAST PLANNER - GLPI</t>
+  </si>
+  <si>
+    <t>No carga información tablero de rendimientos proyecto Provenza Regency (Número de caso 93460)</t>
+  </si>
+  <si>
+    <t>Caso (#93460) - No carga información tablero de rendimientos proyecto Provenza Regency - GLPI</t>
+  </si>
+  <si>
+    <t>Incidencia en el momento de reportar avances (Número de caso 93306)</t>
+  </si>
+  <si>
+    <t>Caso (#93306) - Incidencia en el momento de reportar avances - GLPI</t>
+  </si>
+  <si>
+    <t>Integración para el funcionamiento de grilla para torres altas que se entreguen una sola torre en estapas diferentes (Número de caso 68339)</t>
+  </si>
+  <si>
+    <t>Caso (#68339) - Integración para el funcionamiento de grilla para torres altas que se entreguen unas sola torrre en etapas diferentes - GLPI</t>
+  </si>
+  <si>
+    <t>Acta semanal Country Park (Número de caso 93394)</t>
+  </si>
+  <si>
+    <t>Caso (#93394) - ACTA SEMANAL COUNTRY PARK - GLPI</t>
+  </si>
+  <si>
+    <t>BA-035</t>
+  </si>
+  <si>
+    <t>BA-036</t>
+  </si>
+  <si>
+    <t>BA-037</t>
+  </si>
+  <si>
+    <t>BA-038</t>
+  </si>
+  <si>
+    <t>BA-039</t>
+  </si>
+  <si>
+    <t>BA-040</t>
+  </si>
+  <si>
+    <t>Paola-Daniela</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b33</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b34</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b35</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b36</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b37</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b38</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b39</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b40</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b41</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b42</t>
+  </si>
+  <si>
+    <t>https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b43</t>
+  </si>
+  <si>
+    <t>Herramienta utilizada para la planificación, programación y seguimiento de cronogramas de proyectos, permitiendo analizar rutas críticas, duraciones y secuencia de actividades en apoyo a la gestión de obra.</t>
+  </si>
+  <si>
+    <t>Plataforma colaborativa empleada para la construcción de diagramas, mapas de procesos, sesiones de ideación, talleres LEAN y documentación visual de iniciativas de mejora continua.</t>
+  </si>
+  <si>
+    <t>Plataforma utilizada para registrar, gestionar y dar seguimiento a los requerimientos, incidencias y solicitudes de desarrollo del Área LEAN, facilitando la trazabilidad de las iniciativas.</t>
+  </si>
+  <si>
+    <t>Plataforma de gestión documental utilizada para administrar, consultar y controlar la información técnica de los proyectos, garantizando la trazabilidad de documentos, planos y comunicaciones.</t>
+  </si>
+  <si>
+    <t>Repositorio de apoyo para la consulta de capacitaciones, tutoriales y material audiovisual relacionado con metodologías LEAN, herramientas tecnológicas y procesos internos.</t>
+  </si>
+  <si>
+    <t>Sistema ERP corporativo utilizado para consultar información administrativa y operativa relacionada con proyectos, contratos, presupuestos y demás procesos empresariales que apoyan la gestión del Área LEAN.</t>
+  </si>
+  <si>
+    <t>Herramienta que permite establecer una conexión segura a la red corporativa para acceder de forma remota a aplicaciones, servidores y recursos internos utilizados por el Área LEAN.</t>
+  </si>
+  <si>
+    <t>Extensión de captura de pantalla y grabación de video utilizada para documentar incidencias y registrar evidencias funcionales de Analytics, apoyando el proceso de reporte y seguimiento de desarrollos.</t>
+  </si>
+  <si>
+    <t>Planificación</t>
+  </si>
+  <si>
+    <t>Colaboración</t>
+  </si>
+  <si>
+    <t>Gestion de Requerimientos</t>
+  </si>
+  <si>
+    <t>Gestión Documental</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacitación </t>
+  </si>
+  <si>
+    <t>ERP</t>
+  </si>
+  <si>
+    <t>Captura de Evidencia</t>
+  </si>
+  <si>
+    <t>Accceso Remoto</t>
+  </si>
+  <si>
+    <t>Permalink acuerdos de servicio subidos 2025</t>
+  </si>
+  <si>
+    <t>https://analytics.zoho.com/open-view/1954380000086356866/fd969ba42dcccf08d3ddc846df8aacb76bbb39393f3fdb983c18b28d21853599</t>
+  </si>
+  <si>
+    <t>IND-007</t>
+  </si>
+  <si>
+    <t>Analytics Zoho</t>
+  </si>
+  <si>
+    <t>Dashboard que consolida y visualiza indicadores de desempeño de los proyectos, permitiendo realizar seguimiento al cumplimiento de metas, analizar tendencias y apoyar la toma de decisiones del Área LEAN.</t>
+  </si>
+  <si>
+    <t>Indicador que permite consultar y verificar los acuerdos de servicio cargados en la plataforma mediante enlaces permanentes (permalinks), facilitando el acceso, control y seguimiento de la información por parte del Área LEAN.</t>
+  </si>
+  <si>
+    <t>IND-008</t>
+  </si>
+  <si>
+    <t>Permalink contratos teoricos vs contratos reales</t>
+  </si>
+  <si>
+    <t>Reporte que permite comparar los contratos teóricos definidos en la programación con los contratos reales registrados en el proyecto, facilitando la identificación de diferencias, el seguimiento de la contratación y la validación de la información utilizada por el Área LEAN.</t>
+  </si>
+  <si>
+    <t>https://analytics.zoho.com/open-view/1954380000102979448/88cda4660a1127929863753bced064f2</t>
+  </si>
+  <si>
+    <t>Ingeniero LEAN</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1283,6 +1505,7 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
@@ -1299,12 +1522,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
     <font>
       <b/>
@@ -1370,9 +1587,9 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1384,9 +1601,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1397,22 +1611,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1439,13 +1659,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>16</xdr:row>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>304800</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1487,13 +1707,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>5</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>5</xdr:row>
       <xdr:rowOff>304800</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2166,12 +2386,18 @@
         <v>80</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="150" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>340</v>
+        <v>294</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>345</v>
+        <v>299</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>443</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>33</v>
@@ -2179,20 +2405,26 @@
       <c r="F12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="H12" s="2" t="s">
         <v>35</v>
       </c>
       <c r="I12" s="2"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="135" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>341</v>
+        <v>295</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>346</v>
+        <v>300</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>444</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>33</v>
@@ -2200,20 +2432,26 @@
       <c r="F13" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G13" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="H13" s="3" t="s">
+      <c r="G13" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>35</v>
       </c>
       <c r="I13" s="2"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="135" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>342</v>
+        <v>296</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>347</v>
+        <v>301</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>445</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>33</v>
@@ -2221,20 +2459,26 @@
       <c r="F14" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G14" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="H14" s="3" t="s">
+      <c r="G14" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="H14" s="2" t="s">
         <v>35</v>
       </c>
       <c r="I14" s="2"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="135" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>343</v>
+        <v>297</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>348</v>
+        <v>302</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>446</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>33</v>
@@ -2242,20 +2486,26 @@
       <c r="F15" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G15" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="H15" s="3" t="s">
+      <c r="G15" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="H15" s="2" t="s">
         <v>35</v>
       </c>
       <c r="I15" s="2"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>344</v>
+        <v>298</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>349</v>
+        <v>303</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>447</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>33</v>
@@ -2263,20 +2513,26 @@
       <c r="F16" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G16" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="H16" s="3" t="s">
+      <c r="G16" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="H16" s="2" t="s">
         <v>35</v>
       </c>
       <c r="I16" s="2"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="135" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>351</v>
+        <v>305</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>350</v>
+        <v>304</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>448</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>33</v>
@@ -2284,20 +2540,26 @@
       <c r="F17" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G17" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="H17" s="3" t="s">
+      <c r="G17" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="H17" s="2" t="s">
         <v>35</v>
       </c>
       <c r="I17" s="2"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="135" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>352</v>
+        <v>306</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>353</v>
+        <v>307</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>450</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>33</v>
@@ -2305,20 +2567,26 @@
       <c r="F18" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G18" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="H18" s="3" t="s">
+      <c r="G18" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="H18" s="2" t="s">
         <v>35</v>
       </c>
       <c r="I18" s="2"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>355</v>
+        <v>309</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>354</v>
+        <v>308</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>449</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>33</v>
@@ -2326,29 +2594,29 @@
       <c r="F19" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G19" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="H19" s="3" t="s">
+      <c r="G19" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="H19" s="2" t="s">
         <v>35</v>
       </c>
       <c r="I19" s="2"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="6" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="9" width="25" customWidth="1"/>
+    <col min="1" max="8" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2362,206 +2630,131 @@
         <v>119</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>26</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>120</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>306</v>
+        <v>130</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>131</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>329</v>
+        <v>33</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>328</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>331</v>
+        <v>125</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>332</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="165" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>115</v>
+      <c r="B3" s="8" t="s">
+        <v>326</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>329</v>
+        <v>363</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>328</v>
       </c>
       <c r="G3" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="H3" s="8" t="s">
         <v>328</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>333</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:8" ht="240" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>330</v>
+        <v>292</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>364</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="E4" t="s">
-        <v>329</v>
-      </c>
-      <c r="G4" t="s">
+        <v>365</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>366</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>328</v>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="9" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="G4" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="345" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="B5" t="s">
-        <v>109</v>
+        <v>293</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>368</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="E5" t="s">
-        <v>329</v>
-      </c>
-      <c r="G5" t="s">
+        <v>367</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>366</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>328</v>
       </c>
-      <c r="H5" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="I5" s="9" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="B6" t="s">
-        <v>111</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="E6" t="s">
-        <v>329</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="G5" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="H5" s="8" t="s">
         <v>328</v>
       </c>
-      <c r="H6" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="I6" s="9" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="E7" t="s">
-        <v>329</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>374</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
-        <v>372</v>
-      </c>
-      <c r="D9" t="s">
-        <v>373</v>
-      </c>
-      <c r="E9" t="s">
-        <v>33</v>
-      </c>
-      <c r="F9" t="s">
-        <v>374</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>125</v>
-      </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="6" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="H2" r:id="rId1" location="P163/itemdetails/I102" xr:uid="{4F14EE80-AC72-4FD9-AD96-DF8C921FE23E}"/>
-  </hyperlinks>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{124371BC-E72D-4ACB-81AC-BC0F07668931}">
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
@@ -2597,383 +2790,903 @@
       <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="9" t="s">
         <v>6</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>277</v>
+        <v>238</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>90</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>278</v>
+        <v>239</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+        <v>286</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>280</v>
+        <v>241</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>90</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>281</v>
+        <v>242</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>325</v>
+        <v>286</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>370</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>282</v>
+        <v>243</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>90</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>283</v>
+        <v>244</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+        <v>286</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>284</v>
+        <v>245</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>98</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>285</v>
+        <v>246</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>287</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>286</v>
+        <v>247</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>102</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>287</v>
+        <v>248</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+        <v>288</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>288</v>
+        <v>249</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>103</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>289</v>
+        <v>250</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>288</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>290</v>
+        <v>251</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>92</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>291</v>
+        <v>252</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+        <v>286</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>292</v>
+        <v>253</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>94</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>293</v>
+        <v>254</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>286</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>294</v>
+        <v>255</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>97</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>295</v>
+        <v>256</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+        <v>287</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>296</v>
+        <v>257</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>100</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>297</v>
+        <v>258</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>288</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>298</v>
+        <v>259</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>104</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>299</v>
+        <v>260</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>288</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>300</v>
+        <v>261</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>105</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>301</v>
+        <v>262</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>288</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>302</v>
+        <v>263</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>106</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>303</v>
+        <v>264</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+        <v>288</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>304</v>
+        <v>265</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>107</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>305</v>
+        <v>266</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+        <v>288</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>309</v>
+        <v>357</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>93</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>310</v>
+        <v>271</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>286</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>311</v>
+        <v>358</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>99</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>312</v>
+        <v>273</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+        <v>287</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>313</v>
+        <v>270</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>96</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>314</v>
+        <v>275</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>287</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>315</v>
+        <v>272</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>101</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>316</v>
+        <v>277</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+        <v>288</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>317</v>
+        <v>274</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>91</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>318</v>
+        <v>279</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>240</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>319</v>
+        <v>276</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>95</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>320</v>
+        <v>281</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+        <v>240</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>321</v>
+        <v>278</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>109</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>322</v>
+        <v>283</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>268</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>323</v>
+        <v>280</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>111</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>324</v>
+        <v>285</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>307</v>
+        <v>268</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="I24" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="I25" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>291</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="G26" t="s">
+        <v>289</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>393</v>
+      </c>
+      <c r="I26" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="B27" t="s">
+        <v>109</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="G27" t="s">
+        <v>289</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>394</v>
+      </c>
+      <c r="I27" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="B28" t="s">
+        <v>111</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="G28" t="s">
+        <v>289</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="I28" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="I29" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>432</v>
+      </c>
+      <c r="I30" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="B31" t="s">
+        <v>398</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="B32" t="s">
+        <v>398</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="G32" t="s">
+        <v>289</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="I32" t="s">
+        <v>401</v>
+      </c>
+      <c r="J32" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="B33" t="s">
+        <v>398</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="G33" t="s">
+        <v>289</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="I33" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="B34" t="s">
+        <v>405</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="B35" t="s">
+        <v>414</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="G35" t="s">
+        <v>289</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="I35" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="B36" t="s">
+        <v>416</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="G36" t="s">
+        <v>289</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="I36" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="B37" t="s">
+        <v>418</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="G37" t="s">
+        <v>289</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>439</v>
+      </c>
+      <c r="I37" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="B38" t="s">
+        <v>420</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="G38" t="s">
+        <v>289</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>440</v>
+      </c>
+      <c r="I38" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="B39" t="s">
+        <v>422</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="G39" t="s">
+        <v>289</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>441</v>
+      </c>
+      <c r="I39" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B40" t="s">
+        <v>424</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="G40" t="s">
+        <v>289</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>442</v>
+      </c>
+      <c r="I40" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{CBBFCFAD-F2B4-49E6-AFA2-A2E8E2BEFE02}"/>
+    <hyperlink ref="H3:H29" r:id="rId2" display="https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b5" xr:uid="{B39A16E9-AB55-4A33-AF19-64F1A9B41477}"/>
+    <hyperlink ref="H30:H40" r:id="rId3" display="https://app.notion.com/p/22bd59e7f3bc811886c3f9cd5df7287c?v=22bd59e7f3bc8148a84a000cc9f601b5" xr:uid="{AC1F786A-C574-4F44-A7A1-294557B49834}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="8" width="25" customWidth="1"/>
@@ -3076,6 +3789,9 @@
       <c r="F4" s="2" t="s">
         <v>137</v>
       </c>
+      <c r="G4" t="s">
+        <v>154</v>
+      </c>
       <c r="H4" s="2" t="s">
         <v>146</v>
       </c>
@@ -3111,7 +3827,7 @@
         <v>151</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>377</v>
+        <v>331</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>30</v>
@@ -3132,16 +3848,19 @@
         <v>153</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="135" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>376</v>
+        <v>330</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>375</v>
+        <v>329</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>30</v>
       </c>
+      <c r="D7" s="2" t="s">
+        <v>463</v>
+      </c>
       <c r="E7" s="2" t="s">
         <v>33</v>
       </c>
@@ -3152,11 +3871,61 @@
         <v>154</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>378</v>
+        <v>332</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="165" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="210" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>468</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="6" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="G8" r:id="rId1" xr:uid="{3DE1C176-35E1-43D9-ACB2-74C19F9566B0}"/>
+    <hyperlink ref="G9" r:id="rId2" xr:uid="{855EDAB8-B1EA-4B35-ABA0-9BBA4A35E2E4}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3211,163 +3980,166 @@
       <c r="F2" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G2" s="5" t="s">
-        <v>160</v>
-      </c>
+      <c r="G2" s="16"/>
     </row>
     <row r="3" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>162</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>163</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>166</v>
+      <c r="G3" s="17" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>169</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>172</v>
+        <v>169</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>178</v>
+        <v>174</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>184</v>
+        <v>179</v>
+      </c>
+      <c r="G6" s="17" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>190</v>
+        <v>184</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>196</v>
-      </c>
+        <v>189</v>
+      </c>
+      <c r="G8" s="2"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G3" r:id="rId1" xr:uid="{E450CA4A-B2D1-4690-B3E1-010CCC902B44}"/>
+    <hyperlink ref="G6" r:id="rId2" xr:uid="{95B4B31C-CB0B-4481-8BDB-D15000630CDB}"/>
+    <hyperlink ref="G4" r:id="rId3" xr:uid="{1304D265-C734-41FD-B0DC-79EE4DF3EB3C}"/>
+    <hyperlink ref="G5" r:id="rId4" xr:uid="{7859DA98-00F2-428D-8A15-DBB023397F25}"/>
+    <hyperlink ref="G7" r:id="rId5" xr:uid="{0F00771F-5197-40C4-8FA1-598441B6B712}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing r:id="rId1"/>
+  <legacyDrawing r:id="rId6"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="7" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3390,444 +4162,188 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>205</v>
+        <v>335</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>197</v>
+        <v>333</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>206</v>
+        <v>192</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="G2" s="6">
-        <v>46216</v>
-      </c>
-      <c r="L2" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>206</v>
+      <c r="E2" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>311</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>313</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>191</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="G3" s="6">
-        <v>46216</v>
-      </c>
-      <c r="L3" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>206</v>
+        <v>314</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>312</v>
+      </c>
+      <c r="G3" s="5">
+        <v>46097</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>315</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>316</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>190</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="G4" s="6">
-        <v>46216</v>
-      </c>
-      <c r="L4" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="E4" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="G4" s="5">
+        <v>45757</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>212</v>
+        <v>338</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>213</v>
+        <v>337</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>214</v>
+        <v>339</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="G5" s="6">
-        <v>46216</v>
-      </c>
-      <c r="L5" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>336</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>214</v>
+        <v>345</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>340</v>
+      </c>
+      <c r="C6" t="s">
+        <v>7</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="G6" s="6">
-        <v>46216</v>
-      </c>
-      <c r="L6" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="E6" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="F6" t="s">
+        <v>342</v>
+      </c>
+      <c r="G6" s="5">
+        <v>44697</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>218</v>
+        <v>346</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>343</v>
+      </c>
+      <c r="C7" t="s">
+        <v>7</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="G7" s="6">
-        <v>46216</v>
-      </c>
-      <c r="L7" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="E7" s="13" t="s">
+        <v>344</v>
+      </c>
+      <c r="F7" t="s">
+        <v>342</v>
+      </c>
+      <c r="G7" s="5">
+        <v>44697</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>221</v>
+        <v>347</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>349</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>222</v>
+        <v>7</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>219</v>
+      <c r="E8" s="6" t="s">
+        <v>344</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="G8" s="6">
-        <v>46216</v>
-      </c>
-      <c r="L8" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="G9" s="6">
-        <v>46216</v>
-      </c>
-      <c r="L9" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="G10" s="6">
-        <v>46216</v>
-      </c>
-      <c r="L10" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="G11" s="6">
-        <v>46216</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>381</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>379</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>380</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>330</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="75" x14ac:dyDescent="0.25">
-      <c r="A13" s="13" t="s">
-        <v>357</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>359</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>218</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>358</v>
-      </c>
-      <c r="G13" s="6">
-        <v>46097</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="75" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
-        <v>361</v>
-      </c>
-      <c r="B14" s="16" t="s">
-        <v>362</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>214</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>363</v>
-      </c>
-      <c r="F14" s="13" t="s">
-        <v>356</v>
-      </c>
-      <c r="G14" s="6">
+        <v>348</v>
+      </c>
+      <c r="G8" s="5">
         <v>45757</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>385</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>382</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>330</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="75" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>386</v>
-      </c>
-      <c r="C16" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>387</v>
-      </c>
-      <c r="F16" t="s">
-        <v>388</v>
-      </c>
-      <c r="G16" s="6">
-        <v>44697</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>389</v>
-      </c>
-      <c r="C17" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E17" s="14" t="s">
-        <v>390</v>
-      </c>
-      <c r="F17" t="s">
-        <v>388</v>
-      </c>
-      <c r="G17" s="6">
-        <v>44697</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>395</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>394</v>
-      </c>
-      <c r="G18" s="6">
-        <v>45757</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E19" s="14"/>
-    </row>
-    <row r="22" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="15"/>
-      <c r="B22" s="15"/>
-    </row>
-    <row r="23" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="15"/>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E9" s="13"/>
+    </row>
+    <row r="12" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
+    </row>
+    <row r="13" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="14"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="6" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="E12" r:id="rId1" xr:uid="{CD1E00D1-0B72-42F3-80DA-BD697F689749}"/>
-    <hyperlink ref="E15" r:id="rId2" xr:uid="{BE2AE314-3341-4469-ADFD-A92FCDCAD2AD}"/>
-    <hyperlink ref="B18" r:id="rId3" display="https://us1.aconex.com/rsrc/20260702.0843/es_ES_DOC/document/view/index.html?ControlledDocument_ID=1353331688403523199&amp;ControlledDocument_projectID=1207968420&amp;VIEW_CD_RETURN_URL=%2FSearchControlledDoc%3FSESSION_SAVE_DOCUMENTNO%3D%26SESSION_SAVE_TITLE%3D%2B%26SESSION_SAVE_REVISION%3D%2B%26SESSION_SAVE_STATUS%3D0%26SESSION_SAVE_TYPE%3D0%26SESSION_SAVE_DISCIPLINE%3Dnull%26SESSION_CREATION_DATE%3Dnull%26SESSION_REVISION_DATE%3Dnull%26SESSION_SAVE_REVIEW_DATE%3Dnull%26SESSION_SAVE_REVIEWED_DATE%3Dnull%26SESSION_SAVE_AUTHOR%3Dnull%26SESSION_SAVE_FILETYPE%3Dnull%26SESSION_REFERENCE%3Dnull%26SESSION_SAVE_FOLDER_PATH%3D%26SESSION_SAVE_ALL_REVS%3Dnull%26SESSION_SAVE_SORT_DIR%3DASC%26SESSION_SAVE_SORT_FIELD%3Ddocno%26SESSION_SHARED_TO%3D-1%26SESSION_LINKED_TO_PUBLIC%3D0" xr:uid="{B33F7C5F-686F-4168-AEFA-38B03829F34C}"/>
-    <hyperlink ref="E18" r:id="rId4" display="https://us1.aconex.com/ViewDoc?trackingid=1353331688098790961&amp;projectid=1207968420&amp;cversion=1&amp;tab=0" xr:uid="{3A60C185-9CFD-414E-8CB5-584B4E40E318}"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{CD1E00D1-0B72-42F3-80DA-BD697F689749}"/>
+    <hyperlink ref="E5" r:id="rId2" xr:uid="{BE2AE314-3341-4469-ADFD-A92FCDCAD2AD}"/>
+    <hyperlink ref="B8" r:id="rId3" display="https://us1.aconex.com/rsrc/20260702.0843/es_ES_DOC/document/view/index.html?ControlledDocument_ID=1353331688403523199&amp;ControlledDocument_projectID=1207968420&amp;VIEW_CD_RETURN_URL=%2FSearchControlledDoc%3FSESSION_SAVE_DOCUMENTNO%3D%26SESSION_SAVE_TITLE%3D%2B%26SESSION_SAVE_REVISION%3D%2B%26SESSION_SAVE_STATUS%3D0%26SESSION_SAVE_TYPE%3D0%26SESSION_SAVE_DISCIPLINE%3Dnull%26SESSION_CREATION_DATE%3Dnull%26SESSION_REVISION_DATE%3Dnull%26SESSION_SAVE_REVIEW_DATE%3Dnull%26SESSION_SAVE_REVIEWED_DATE%3Dnull%26SESSION_SAVE_AUTHOR%3Dnull%26SESSION_SAVE_FILETYPE%3Dnull%26SESSION_REFERENCE%3Dnull%26SESSION_SAVE_FOLDER_PATH%3D%26SESSION_SAVE_ALL_REVS%3Dnull%26SESSION_SAVE_SORT_DIR%3DASC%26SESSION_SAVE_SORT_FIELD%3Ddocno%26SESSION_SHARED_TO%3D-1%26SESSION_LINKED_TO_PUBLIC%3D0" xr:uid="{B33F7C5F-686F-4168-AEFA-38B03829F34C}"/>
+    <hyperlink ref="E8" r:id="rId4" xr:uid="{3A60C185-9CFD-414E-8CB5-584B4E40E318}"/>
+    <hyperlink ref="E4" r:id="rId5" xr:uid="{F6E3CF0D-17C9-4F23-A241-03FF5ABD0FEF}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId6"/>
 </worksheet>
 </file>
 
@@ -3851,7 +4367,7 @@
         <v>22</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>235</v>
+        <v>196</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>23</v>
@@ -3865,358 +4381,358 @@
     </row>
     <row r="2" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>236</v>
+        <v>197</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>237</v>
+        <v>198</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>239</v>
+        <v>193</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>200</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>232</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>240</v>
+        <v>201</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>233</v>
+        <v>469</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>241</v>
+        <v>202</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>242</v>
+        <v>195</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>203</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>232</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>243</v>
+        <v>204</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>245</v>
+        <v>206</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>241</v>
+        <v>202</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>246</v>
+        <v>210</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>207</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>248</v>
+        <v>209</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>244</v>
+        <v>205</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>245</v>
+        <v>206</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>241</v>
+        <v>202</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>247</v>
+        <v>210</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>208</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>248</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
-        <v>233</v>
+        <v>469</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="E6" s="7"/>
+        <v>195</v>
+      </c>
+      <c r="E6" s="6"/>
       <c r="F6" s="2" t="s">
-        <v>232</v>
+        <v>194</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>250</v>
+        <v>211</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>364</v>
+        <v>318</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>251</v>
+        <v>210</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>212</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>248</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>252</v>
+        <v>213</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>364</v>
+        <v>318</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>253</v>
+        <v>210</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>214</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>248</v>
+        <v>209</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>365</v>
+        <v>319</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>364</v>
+        <v>318</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>366</v>
+        <v>210</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>320</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>248</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>254</v>
+        <v>215</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A12" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
+        <v>323</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="B18" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>265</v>
-      </c>
-      <c r="F10" s="2" t="s">
+      <c r="C18" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="E18" s="7" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
-        <v>256</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
-        <v>258</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>259</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
-        <v>260</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>261</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
-        <v>262</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>263</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
-        <v>367</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>371</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>368</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
-        <v>369</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>371</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>370</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
-        <v>266</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>270</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>269</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
-        <v>272</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>270</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>271</v>
-      </c>
       <c r="F18" s="2" t="s">
-        <v>268</v>
+        <v>229</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A19" s="9" t="s">
-        <v>275</v>
+      <c r="A19" s="8" t="s">
+        <v>236</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>274</v>
+        <v>235</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>241</v>
+        <v>202</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>270</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>276</v>
+        <v>231</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>237</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>268</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>